<commit_message>
Fix workflow permissions and add Kai Fong's May 22 workout update
</commit_message>
<xml_diff>
--- a/Reports/Members/Kai Fong_Activity_Report.xlsx
+++ b/Reports/Members/Kai Fong_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -627,6 +627,53 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5/22/2026 8:02:19</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kai Fong</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3.99</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -675,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17.42</v>
+        <v>21.41</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -745,7 +792,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.82</v>
+        <v>22.81</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>

</xml_diff>